<commit_message>
Update configuration for FirmenABC scraping and enhance search fallback features
- Changed base and start URLs to target FirmenABC directory.
- Added new parameters for saving data and timeout settings.
- Updated detail page URL pattern to accommodate new structure.
- Enhanced website field selectors to capture additional website links.
- Enabled search fallback for incomplete detail pages with configurable options.
- Modified HTTP headers for improved request compatibility.
</commit_message>
<xml_diff>
--- a/business_listings.xlsx
+++ b/business_listings.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +55,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,11 +424,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
@@ -425,52 +436,230 @@
     <col width="5" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>UID</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Registry Number</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Credit Reference</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Scraped At</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Data Quality (%)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Enriched</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/ayna-personalvermittlung-e-u_BBcgl</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Ayna Personalvermittlung E U</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24T16:03:18Z</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/glaubenkranz-e-u_GXkR</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Glaubenkranz E U</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24T16:05:07Z</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/mick-michael-denkmal-fassaden-u-gebaeudereinigung-meisterbet_BBbMH</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Mick Michael Denkmal Fassaden U Gebaeudereinigung Meisterbet</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24T16:06:52Z</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/hubek-versicherungs-und-finanzservice_MyUP</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Hubek Versicherungs Und Finanzservice</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24T16:08:33Z</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/speedexpress-gebaeudereinigung-gmbh_BBjHb</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Speedexpress Gebaeudereinigung Gmbh</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24T16:10:15Z</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>